<commit_message>
Membenahi beberapa tmapian dan logic fitur bank soal
</commit_message>
<xml_diff>
--- a/file_lain/dummy_bank_soal_bahasa_jawa.xlsx
+++ b/file_lain/dummy_bank_soal_bahasa_jawa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FILE TUGAS AKHIR\~APLIKASI\Website CAT\file_lain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFE974E-FC0A-437F-9837-B43E33E325E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB628C3F-E7CD-4745-B0DA-504AEE347A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Soal" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="289">
   <si>
     <t>Kategori</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Opsi E</t>
   </si>
   <si>
-    <t>Opsi F</t>
-  </si>
-  <si>
     <t>Jawaban</t>
   </si>
   <si>
@@ -428,9 +425,6 @@
     <t>Yang termasuk tingkat tutur (undha-usuk) dalam Bahasa Jawa adalah...</t>
   </si>
   <si>
-    <t>Basa campur</t>
-  </si>
-  <si>
     <t>A,B,C</t>
   </si>
   <si>
@@ -452,18 +446,12 @@
     <t>Suku (krama: kaki)</t>
   </si>
   <si>
-    <t>Pupuk (krama: perut)</t>
-  </si>
-  <si>
     <t>B,D,E</t>
   </si>
   <si>
     <t>Yang termasuk tembang macapat adalah...</t>
   </si>
   <si>
-    <t>Megatruh</t>
-  </si>
-  <si>
     <t>A,B,C,D,E,F</t>
   </si>
   <si>
@@ -485,9 +473,6 @@
     <t>Gamelan</t>
   </si>
   <si>
-    <t>Sinden</t>
-  </si>
-  <si>
     <t>Paribasan Jawa yang mengandung nasihat hidup adalah...</t>
   </si>
   <si>
@@ -521,9 +506,6 @@
     <t>Suluk</t>
   </si>
   <si>
-    <t>Wulang</t>
-  </si>
-  <si>
     <t>A,B,D,E</t>
   </si>
   <si>
@@ -545,9 +527,6 @@
     <t>Menulis surat resmi</t>
   </si>
   <si>
-    <t>Dekorasi</t>
-  </si>
-  <si>
     <t>A,C,D</t>
   </si>
   <si>
@@ -569,9 +548,6 @@
     <t>Reog</t>
   </si>
   <si>
-    <t>Kuda lumping</t>
-  </si>
-  <si>
     <t>Sapaan/sembah dalam Bahasa Jawa krama untuk menyapa orang yang dihormati bisa menggunakan...</t>
   </si>
   <si>
@@ -590,9 +566,6 @@
     <t>Nuwun sewu</t>
   </si>
   <si>
-    <t>Monggo pinarak</t>
-  </si>
-  <si>
     <t>Serat Wulang atau piwulang berisi ajaran tentang...</t>
   </si>
   <si>
@@ -611,9 +584,6 @@
     <t>Kesenian</t>
   </si>
   <si>
-    <t>Kesehatan</t>
-  </si>
-  <si>
     <t>A,B,C,D</t>
   </si>
   <si>
@@ -635,9 +605,6 @@
     <t>Slametan</t>
   </si>
   <si>
-    <t>Sekaten</t>
-  </si>
-  <si>
     <t>Jenis batik menurut teknik/cara pembuatan adalah...</t>
   </si>
   <si>
@@ -668,9 +635,6 @@
     <t>Sadewa</t>
   </si>
   <si>
-    <t>Kresna</t>
-  </si>
-  <si>
     <t>Yang termasuk ungkapan permohonan maaf dalam Bahasa Jawa adalah...</t>
   </si>
   <si>
@@ -702,9 +666,6 @@
   </si>
   <si>
     <t>Hormat kepada orang tua</t>
-  </si>
-  <si>
-    <t>Kejujuran</t>
   </si>
   <si>
     <t>Tentukan benar/salah pernyataan tentang tingkat tutur Bahasa Jawa.</t>
@@ -1303,19 +1264,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="52.83203125" customWidth="1"/>
-    <col min="3" max="6" width="36.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.796875" customWidth="1"/>
+    <col min="2" max="2" width="52.796875" customWidth="1"/>
+    <col min="3" max="6" width="36.796875" customWidth="1"/>
+    <col min="7" max="7" width="22.796875" customWidth="1"/>
+    <col min="8" max="8" width="14.796875" customWidth="1"/>
+    <col min="9" max="9" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1343,1614 +1303,1461 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
       </c>
       <c r="H2" t="s">
         <v>16</v>
       </c>
       <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>299</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
       <c r="I3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>299</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>29</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
       </c>
       <c r="H4" t="s">
         <v>16</v>
       </c>
       <c r="I4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>33</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>34</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>35</v>
-      </c>
-      <c r="G5" t="s">
-        <v>36</v>
       </c>
       <c r="H5" t="s">
         <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>38</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>40</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>42</v>
       </c>
-      <c r="H6" t="s">
-        <v>16</v>
-      </c>
       <c r="I6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B7" t="s">
         <v>43</v>
       </c>
-      <c r="J6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>299</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>45</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>48</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
       </c>
       <c r="I7" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>53</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>54</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>286</v>
+      </c>
+      <c r="B9" t="s">
         <v>55</v>
       </c>
-      <c r="H8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" t="s">
-        <v>43</v>
-      </c>
-      <c r="J8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>299</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>56</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>58</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>59</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>60</v>
-      </c>
-      <c r="G9" t="s">
-        <v>61</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
         <v>62</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>63</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>65</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>66</v>
-      </c>
-      <c r="G10" t="s">
-        <v>67</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
       </c>
       <c r="I10" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
         <v>68</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>69</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>70</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>71</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>72</v>
-      </c>
-      <c r="G11" t="s">
-        <v>73</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
       </c>
       <c r="I11" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" t="s">
         <v>74</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>75</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>76</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>77</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>78</v>
-      </c>
-      <c r="G12" t="s">
-        <v>79</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
       </c>
       <c r="I12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s">
         <v>80</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>81</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>82</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>83</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>84</v>
-      </c>
-      <c r="G13" t="s">
-        <v>85</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
       </c>
       <c r="I13" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" t="s">
         <v>86</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>87</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>88</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>89</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>90</v>
-      </c>
-      <c r="G14" t="s">
-        <v>91</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
       </c>
       <c r="I14" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
         <v>92</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>93</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>94</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>95</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>96</v>
-      </c>
-      <c r="G15" t="s">
-        <v>97</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
       </c>
       <c r="I15" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B16" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" t="s">
         <v>98</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>99</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>100</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>101</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>102</v>
-      </c>
-      <c r="G16" t="s">
-        <v>103</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
       </c>
       <c r="I16" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" t="s">
         <v>104</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>105</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>106</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>107</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>108</v>
-      </c>
-      <c r="G17" t="s">
-        <v>109</v>
       </c>
       <c r="H17" t="s">
         <v>16</v>
       </c>
       <c r="I17" t="s">
-        <v>17</v>
-      </c>
-      <c r="J17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" t="s">
         <v>110</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>111</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>112</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>113</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>114</v>
-      </c>
-      <c r="G18" t="s">
-        <v>115</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
       </c>
       <c r="I18" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" t="s">
         <v>116</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>117</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>118</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>119</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>120</v>
-      </c>
-      <c r="G19" t="s">
-        <v>121</v>
       </c>
       <c r="H19" t="s">
         <v>16</v>
       </c>
       <c r="I19" t="s">
-        <v>17</v>
-      </c>
-      <c r="J19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" t="s">
         <v>122</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>123</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>124</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>125</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>126</v>
-      </c>
-      <c r="G20" t="s">
-        <v>127</v>
       </c>
       <c r="H20" t="s">
         <v>16</v>
       </c>
       <c r="I20" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" t="s">
         <v>128</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>129</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>130</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>131</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>132</v>
-      </c>
-      <c r="G21" t="s">
-        <v>133</v>
       </c>
       <c r="H21" t="s">
         <v>16</v>
       </c>
       <c r="I21" t="s">
-        <v>17</v>
-      </c>
-      <c r="J21" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="B22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" t="s">
         <v>134</v>
       </c>
-      <c r="C22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>287</v>
+      </c>
+      <c r="B23" t="s">
         <v>135</v>
       </c>
-      <c r="I22" t="s">
+      <c r="C23" t="s">
         <v>136</v>
       </c>
-      <c r="J22" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>300</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>137</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>138</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>139</v>
       </c>
-      <c r="E23" t="s">
+      <c r="G23" t="s">
         <v>140</v>
       </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>141</v>
       </c>
-      <c r="G23" t="s">
+      <c r="I23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>287</v>
+      </c>
+      <c r="B24" t="s">
         <v>142</v>
       </c>
-      <c r="H23" t="s">
+      <c r="C24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+      <c r="G24" t="s">
+        <v>41</v>
+      </c>
+      <c r="H24" t="s">
         <v>143</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>287</v>
+      </c>
+      <c r="B25" t="s">
         <v>144</v>
       </c>
-      <c r="J23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>300</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C25" t="s">
         <v>145</v>
       </c>
-      <c r="C24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" t="s">
-        <v>38</v>
-      </c>
-      <c r="G24" t="s">
-        <v>42</v>
-      </c>
-      <c r="H24" t="s">
+      <c r="D25" t="s">
         <v>146</v>
       </c>
-      <c r="I24" t="s">
+      <c r="E25" t="s">
         <v>147</v>
       </c>
-      <c r="J24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>300</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="F25" t="s">
         <v>148</v>
       </c>
-      <c r="C25" t="s">
+      <c r="G25" t="s">
         <v>149</v>
       </c>
-      <c r="D25" t="s">
+      <c r="H25" t="s">
+        <v>143</v>
+      </c>
+      <c r="I25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>287</v>
+      </c>
+      <c r="B26" t="s">
         <v>150</v>
       </c>
-      <c r="E25" t="s">
+      <c r="C26" t="s">
         <v>151</v>
       </c>
-      <c r="F25" t="s">
+      <c r="D26" t="s">
         <v>152</v>
       </c>
-      <c r="G25" t="s">
+      <c r="E26" t="s">
         <v>153</v>
       </c>
-      <c r="H25" t="s">
+      <c r="F26" t="s">
         <v>154</v>
       </c>
-      <c r="I25" t="s">
-        <v>147</v>
-      </c>
-      <c r="J25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>300</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="G26" t="s">
         <v>155</v>
       </c>
-      <c r="C26" t="s">
+      <c r="H26" t="s">
         <v>156</v>
       </c>
-      <c r="D26" t="s">
+      <c r="I26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>287</v>
+      </c>
+      <c r="B27" t="s">
         <v>157</v>
       </c>
-      <c r="E26" t="s">
+      <c r="C27" t="s">
         <v>158</v>
       </c>
-      <c r="F26" t="s">
+      <c r="D27" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" t="s">
+        <v>50</v>
+      </c>
+      <c r="F27" t="s">
         <v>159</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G27" t="s">
         <v>160</v>
       </c>
-      <c r="H26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="H27" t="s">
         <v>161</v>
       </c>
-      <c r="J26" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>300</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="I27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>287</v>
+      </c>
+      <c r="B28" t="s">
         <v>162</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>163</v>
       </c>
-      <c r="D27" t="s">
-        <v>52</v>
-      </c>
-      <c r="E27" t="s">
-        <v>51</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="D28" t="s">
         <v>164</v>
       </c>
-      <c r="G27" t="s">
+      <c r="E28" t="s">
         <v>165</v>
       </c>
-      <c r="H27" t="s">
+      <c r="F28" t="s">
         <v>166</v>
       </c>
-      <c r="I27" t="s">
+      <c r="G28" t="s">
         <v>167</v>
       </c>
-      <c r="J27" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>300</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="H28" t="s">
         <v>168</v>
       </c>
-      <c r="C28" t="s">
+      <c r="I28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>287</v>
+      </c>
+      <c r="B29" t="s">
         <v>169</v>
       </c>
-      <c r="D28" t="s">
+      <c r="C29" t="s">
         <v>170</v>
       </c>
-      <c r="E28" t="s">
+      <c r="D29" t="s">
         <v>171</v>
       </c>
-      <c r="F28" t="s">
+      <c r="E29" t="s">
         <v>172</v>
       </c>
-      <c r="G28" t="s">
+      <c r="F29" t="s">
         <v>173</v>
       </c>
-      <c r="H28" t="s">
+      <c r="G29" t="s">
         <v>174</v>
       </c>
-      <c r="I28" t="s">
+      <c r="H29" t="s">
+        <v>143</v>
+      </c>
+      <c r="I29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>287</v>
+      </c>
+      <c r="B30" t="s">
         <v>175</v>
       </c>
-      <c r="J28" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>300</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C30" t="s">
         <v>176</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D30" t="s">
         <v>177</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E30" t="s">
         <v>178</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F30" t="s">
         <v>179</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G30" t="s">
         <v>180</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H30" t="s">
+        <v>156</v>
+      </c>
+      <c r="I30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>287</v>
+      </c>
+      <c r="B31" t="s">
         <v>181</v>
       </c>
-      <c r="H29" t="s">
+      <c r="C31" t="s">
         <v>182</v>
       </c>
-      <c r="I29" t="s">
-        <v>147</v>
-      </c>
-      <c r="J29" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>300</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="D31" t="s">
         <v>183</v>
       </c>
-      <c r="C30" t="s">
+      <c r="E31" t="s">
         <v>184</v>
       </c>
-      <c r="D30" t="s">
+      <c r="F31" t="s">
         <v>185</v>
       </c>
-      <c r="E30" t="s">
+      <c r="G31" t="s">
         <v>186</v>
       </c>
-      <c r="F30" t="s">
+      <c r="H31" t="s">
         <v>187</v>
       </c>
-      <c r="G30" t="s">
+      <c r="I31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>287</v>
+      </c>
+      <c r="B32" t="s">
         <v>188</v>
       </c>
-      <c r="H30" t="s">
+      <c r="C32" t="s">
         <v>189</v>
       </c>
-      <c r="I30" t="s">
-        <v>161</v>
-      </c>
-      <c r="J30" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>300</v>
-      </c>
-      <c r="B31" t="s">
+      <c r="D32" t="s">
         <v>190</v>
       </c>
-      <c r="C31" t="s">
+      <c r="E32" t="s">
         <v>191</v>
       </c>
-      <c r="D31" t="s">
+      <c r="F32" t="s">
         <v>192</v>
       </c>
-      <c r="E31" t="s">
+      <c r="G32" t="s">
         <v>193</v>
       </c>
-      <c r="F31" t="s">
+      <c r="H32" t="s">
+        <v>156</v>
+      </c>
+      <c r="I32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>287</v>
+      </c>
+      <c r="B33" t="s">
         <v>194</v>
       </c>
-      <c r="G31" t="s">
+      <c r="C33" t="s">
         <v>195</v>
       </c>
-      <c r="H31" t="s">
+      <c r="D33" t="s">
+        <v>119</v>
+      </c>
+      <c r="E33" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" t="s">
+        <v>116</v>
+      </c>
+      <c r="G33" t="s">
         <v>196</v>
       </c>
-      <c r="I31" t="s">
+      <c r="H33" t="s">
         <v>197</v>
       </c>
-      <c r="J31" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>300</v>
-      </c>
-      <c r="B32" t="s">
+      <c r="I33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>287</v>
+      </c>
+      <c r="B34" t="s">
         <v>198</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C34" t="s">
         <v>199</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D34" t="s">
         <v>200</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E34" t="s">
         <v>201</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F34" t="s">
         <v>202</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G34" t="s">
         <v>203</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H34" t="s">
+        <v>156</v>
+      </c>
+      <c r="I34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>287</v>
+      </c>
+      <c r="B35" t="s">
         <v>204</v>
       </c>
-      <c r="I32" t="s">
-        <v>161</v>
-      </c>
-      <c r="J32" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>300</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="C35" t="s">
+        <v>180</v>
+      </c>
+      <c r="D35" t="s">
+        <v>178</v>
+      </c>
+      <c r="E35" t="s">
         <v>205</v>
       </c>
-      <c r="C33" t="s">
+      <c r="F35" t="s">
         <v>206</v>
       </c>
-      <c r="D33" t="s">
-        <v>120</v>
-      </c>
-      <c r="E33" t="s">
-        <v>118</v>
-      </c>
-      <c r="F33" t="s">
-        <v>117</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="G35" t="s">
         <v>207</v>
       </c>
-      <c r="H33" t="s">
-        <v>121</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="H35" t="s">
         <v>208</v>
       </c>
-      <c r="J33" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>300</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="I35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>287</v>
+      </c>
+      <c r="B36" t="s">
         <v>209</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C36" t="s">
         <v>210</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D36" t="s">
         <v>211</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E36" t="s">
         <v>212</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F36" t="s">
         <v>213</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G36" t="s">
         <v>214</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H36" t="s">
+        <v>143</v>
+      </c>
+      <c r="I36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>288</v>
+      </c>
+      <c r="B37" t="s">
         <v>215</v>
       </c>
-      <c r="I34" t="s">
-        <v>161</v>
-      </c>
-      <c r="J34" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>300</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="C37" t="s">
         <v>216</v>
       </c>
-      <c r="C35" t="s">
-        <v>188</v>
-      </c>
-      <c r="D35" t="s">
-        <v>186</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="D37" t="s">
         <v>217</v>
       </c>
-      <c r="F35" t="s">
+      <c r="E37" t="s">
         <v>218</v>
       </c>
-      <c r="G35" t="s">
+      <c r="F37" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
         <v>219</v>
       </c>
-      <c r="H35" t="s">
-        <v>185</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="I37" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>288</v>
+      </c>
+      <c r="B38" t="s">
         <v>220</v>
       </c>
-      <c r="J35" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>300</v>
-      </c>
-      <c r="B36" t="s">
+      <c r="C38" t="s">
         <v>221</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D38" t="s">
         <v>222</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E38" t="s">
         <v>223</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F38" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
+        <v>219</v>
+      </c>
+      <c r="I38" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>288</v>
+      </c>
+      <c r="B39" t="s">
         <v>224</v>
       </c>
-      <c r="F36" t="s">
+      <c r="C39" t="s">
         <v>225</v>
       </c>
-      <c r="G36" t="s">
+      <c r="D39" t="s">
         <v>226</v>
       </c>
-      <c r="H36" t="s">
+      <c r="E39" t="s">
         <v>227</v>
       </c>
-      <c r="I36" t="s">
-        <v>147</v>
-      </c>
-      <c r="J36" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>301</v>
-      </c>
-      <c r="B37" t="s">
+      <c r="F39" t="s">
+        <v>15</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
         <v>228</v>
       </c>
-      <c r="C37" t="s">
+      <c r="I39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>288</v>
+      </c>
+      <c r="B40" t="s">
         <v>229</v>
       </c>
-      <c r="D37" t="s">
+      <c r="C40" t="s">
         <v>230</v>
       </c>
-      <c r="E37" t="s">
+      <c r="D40" t="s">
         <v>231</v>
       </c>
-      <c r="F37" t="s">
-        <v>16</v>
-      </c>
-      <c r="G37" t="s">
-        <v>16</v>
-      </c>
-      <c r="H37" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" t="s">
+      <c r="E40" t="s">
         <v>232</v>
       </c>
-      <c r="J37" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>301</v>
-      </c>
-      <c r="B38" t="s">
+      <c r="F40" t="s">
+        <v>15</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
+        <v>219</v>
+      </c>
+      <c r="I40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>288</v>
+      </c>
+      <c r="B41" t="s">
         <v>233</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C41" t="s">
         <v>234</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D41" t="s">
         <v>235</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E41" t="s">
         <v>236</v>
       </c>
-      <c r="F38" t="s">
-        <v>16</v>
-      </c>
-      <c r="G38" t="s">
-        <v>16</v>
-      </c>
-      <c r="H38" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" t="s">
-        <v>232</v>
-      </c>
-      <c r="J38" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>301</v>
-      </c>
-      <c r="B39" t="s">
+      <c r="F41" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>228</v>
+      </c>
+      <c r="I41" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>288</v>
+      </c>
+      <c r="B42" t="s">
         <v>237</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C42" t="s">
         <v>238</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D42" t="s">
         <v>239</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E42" t="s">
         <v>240</v>
       </c>
-      <c r="F39" t="s">
-        <v>16</v>
-      </c>
-      <c r="G39" t="s">
-        <v>16</v>
-      </c>
-      <c r="H39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s">
+      <c r="F42" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>228</v>
+      </c>
+      <c r="I42" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>288</v>
+      </c>
+      <c r="B43" t="s">
         <v>241</v>
       </c>
-      <c r="J39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>301</v>
-      </c>
-      <c r="B40" t="s">
+      <c r="C43" t="s">
         <v>242</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D43" t="s">
         <v>243</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E43" t="s">
         <v>244</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F43" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>228</v>
+      </c>
+      <c r="I43" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>288</v>
+      </c>
+      <c r="B44" t="s">
         <v>245</v>
       </c>
-      <c r="F40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" t="s">
-        <v>16</v>
-      </c>
-      <c r="H40" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40" t="s">
-        <v>232</v>
-      </c>
-      <c r="J40" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>301</v>
-      </c>
-      <c r="B41" t="s">
+      <c r="C44" t="s">
         <v>246</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D44" t="s">
         <v>247</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E44" t="s">
         <v>248</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F44" t="s">
+        <v>15</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>219</v>
+      </c>
+      <c r="I44" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>288</v>
+      </c>
+      <c r="B45" t="s">
         <v>249</v>
       </c>
-      <c r="F41" t="s">
-        <v>16</v>
-      </c>
-      <c r="G41" t="s">
-        <v>16</v>
-      </c>
-      <c r="H41" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" t="s">
-        <v>241</v>
-      </c>
-      <c r="J41" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>301</v>
-      </c>
-      <c r="B42" t="s">
+      <c r="C45" t="s">
         <v>250</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D45" t="s">
         <v>251</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E45" t="s">
         <v>252</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F45" t="s">
+        <v>15</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" t="s">
+        <v>219</v>
+      </c>
+      <c r="I45" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>288</v>
+      </c>
+      <c r="B46" t="s">
         <v>253</v>
       </c>
-      <c r="F42" t="s">
-        <v>16</v>
-      </c>
-      <c r="G42" t="s">
-        <v>16</v>
-      </c>
-      <c r="H42" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" t="s">
-        <v>241</v>
-      </c>
-      <c r="J42" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>301</v>
-      </c>
-      <c r="B43" t="s">
+      <c r="C46" t="s">
         <v>254</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D46" t="s">
         <v>255</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E46" t="s">
         <v>256</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F46" t="s">
+        <v>15</v>
+      </c>
+      <c r="G46" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" t="s">
+        <v>228</v>
+      </c>
+      <c r="I46" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>288</v>
+      </c>
+      <c r="B47" t="s">
         <v>257</v>
       </c>
-      <c r="F43" t="s">
-        <v>16</v>
-      </c>
-      <c r="G43" t="s">
-        <v>16</v>
-      </c>
-      <c r="H43" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" t="s">
-        <v>241</v>
-      </c>
-      <c r="J43" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>301</v>
-      </c>
-      <c r="B44" t="s">
+      <c r="C47" t="s">
         <v>258</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D47" t="s">
         <v>259</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E47" t="s">
         <v>260</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F47" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>228</v>
+      </c>
+      <c r="I47" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>288</v>
+      </c>
+      <c r="B48" t="s">
         <v>261</v>
       </c>
-      <c r="F44" t="s">
-        <v>16</v>
-      </c>
-      <c r="G44" t="s">
-        <v>16</v>
-      </c>
-      <c r="H44" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" t="s">
-        <v>232</v>
-      </c>
-      <c r="J44" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>301</v>
-      </c>
-      <c r="B45" t="s">
+      <c r="C48" t="s">
         <v>262</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D48" t="s">
         <v>263</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E48" t="s">
         <v>264</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F48" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>219</v>
+      </c>
+      <c r="I48" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>288</v>
+      </c>
+      <c r="B49" t="s">
         <v>265</v>
       </c>
-      <c r="F45" t="s">
-        <v>16</v>
-      </c>
-      <c r="G45" t="s">
-        <v>16</v>
-      </c>
-      <c r="H45" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" t="s">
-        <v>232</v>
-      </c>
-      <c r="J45" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>301</v>
-      </c>
-      <c r="B46" t="s">
+      <c r="C49" t="s">
         <v>266</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D49" t="s">
         <v>267</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E49" t="s">
         <v>268</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F49" t="s">
+        <v>15</v>
+      </c>
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
+        <v>219</v>
+      </c>
+      <c r="I49" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>288</v>
+      </c>
+      <c r="B50" t="s">
         <v>269</v>
       </c>
-      <c r="F46" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" t="s">
-        <v>16</v>
-      </c>
-      <c r="H46" t="s">
-        <v>16</v>
-      </c>
-      <c r="I46" t="s">
-        <v>241</v>
-      </c>
-      <c r="J46" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>301</v>
-      </c>
-      <c r="B47" t="s">
+      <c r="C50" t="s">
         <v>270</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D50" t="s">
         <v>271</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E50" t="s">
         <v>272</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F50" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
+        <v>228</v>
+      </c>
+      <c r="I50" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>288</v>
+      </c>
+      <c r="B51" t="s">
         <v>273</v>
       </c>
-      <c r="F47" t="s">
-        <v>16</v>
-      </c>
-      <c r="G47" t="s">
-        <v>16</v>
-      </c>
-      <c r="H47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" t="s">
-        <v>241</v>
-      </c>
-      <c r="J47" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>301</v>
-      </c>
-      <c r="B48" t="s">
+      <c r="C51" t="s">
         <v>274</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D51" t="s">
         <v>275</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E51" t="s">
         <v>276</v>
       </c>
-      <c r="E48" t="s">
-        <v>277</v>
-      </c>
-      <c r="F48" t="s">
-        <v>16</v>
-      </c>
-      <c r="G48" t="s">
-        <v>16</v>
-      </c>
-      <c r="H48" t="s">
-        <v>16</v>
-      </c>
-      <c r="I48" t="s">
-        <v>232</v>
-      </c>
-      <c r="J48" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>301</v>
-      </c>
-      <c r="B49" t="s">
-        <v>278</v>
-      </c>
-      <c r="C49" t="s">
-        <v>279</v>
-      </c>
-      <c r="D49" t="s">
-        <v>280</v>
-      </c>
-      <c r="E49" t="s">
-        <v>281</v>
-      </c>
-      <c r="F49" t="s">
-        <v>16</v>
-      </c>
-      <c r="G49" t="s">
-        <v>16</v>
-      </c>
-      <c r="H49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" t="s">
-        <v>232</v>
-      </c>
-      <c r="J49" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>301</v>
-      </c>
-      <c r="B50" t="s">
-        <v>282</v>
-      </c>
-      <c r="C50" t="s">
-        <v>283</v>
-      </c>
-      <c r="D50" t="s">
-        <v>284</v>
-      </c>
-      <c r="E50" t="s">
-        <v>285</v>
-      </c>
-      <c r="F50" t="s">
-        <v>16</v>
-      </c>
-      <c r="G50" t="s">
-        <v>16</v>
-      </c>
-      <c r="H50" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" t="s">
-        <v>241</v>
-      </c>
-      <c r="J50" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>301</v>
-      </c>
-      <c r="B51" t="s">
-        <v>286</v>
-      </c>
-      <c r="C51" t="s">
-        <v>287</v>
-      </c>
-      <c r="D51" t="s">
-        <v>288</v>
-      </c>
-      <c r="E51" t="s">
-        <v>289</v>
-      </c>
       <c r="F51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H51" t="s">
-        <v>16</v>
+        <v>228</v>
       </c>
       <c r="I51" t="s">
-        <v>241</v>
-      </c>
-      <c r="J51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J1 B51:J51 B2:J2 B3:J3 B4:J4 B5:J5 B6:J6 B7:J7 B8:J8 B9:J9 B10:J10 B11:J11 B12:J12 B13:J13 B14:J14 B15:J15 B16:J16 B17:J17 B18:J18 B19:J19 B20:J20 B21:J21 B22:J22 B23:J23 B24:J24 B25:J25 B26:J26 B27:J27 B28:J28 B29:J29 B30:J30 B31:J31 B32:J32 B33:J33 B34:J34 B35:J35 B36:J36 B37:J37 B38:J38 B39:J39 B40:J40 B41:J41 B42:J42 B43:J43 B44:J44 B45:J45 B46:J46 B47:J47 B48:J48 B49:J49 B50:J50" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G1 B51:G51 B2:G2 B3:G3 B4:G4 B5:G5 B6:G6 B7:G7 B8:G8 B9:G9 B10:G10 B11:G11 B12:G12 B13:G13 B14:G14 B15:G15 B16:G16 B17:G17 B18:G18 B19:G19 B20:G20 B21:G21 B22:G22 B23:G23 B24:G24 B25:G25 B26:G26 B27:G27 B28:G28 B29:G29 B30:G30 B31:G31 B32:G32 B33:G33 B34:G34 B35:G35 B36:G36 B37:G37 B38:G38 B39:G39 B40:G40 B41:G41 B42:G42 B43:G43 B44:G44 B45:G45 B46:G46 B47:G47 B48:G48 B49:G49 B50:G50 H1:I1 H51:I51 H2:I2 H3:I3 H4:I4 H5:I5 H6:I6 H7:I7 H8:I8 H9:I9 H10:I10 H11:I11 H12:I12 H13:I13 H14:I14 H15:I15 H16:I16 H17:I17 H18:I18 H19:I19 H20:I20 H21:I21 H22:I22 H23:I23 H24:I24 H25:I25 H26:I26 H27:I27 H28:I28 H29:I29 H30:I30 H31:I31 H32:I32 H33:I33 H34:I34 H35:I35 H36:I36 H37:I37 H38:I38 H39:I39 H40:I40 H41:I41 H42:I42 H43:I43 H44:I44 H45:I45 H46:I46 H47:I47 H48:I48 H49:I49 H50:I50" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2958,65 +2765,65 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50.83203125" customWidth="1"/>
-    <col min="2" max="2" width="75.83203125" customWidth="1"/>
+    <col min="1" max="1" width="50.796875" customWidth="1"/>
+    <col min="2" max="2" width="75.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="B6" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
       <c r="B8" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>298</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>